<commit_message>
AFTER TANGENT X OR H
</commit_message>
<xml_diff>
--- a/LİNKLER_Ademden.xlsx
+++ b/LİNKLER_Ademden.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mADEMatik\Desktop\GEO12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0D45B0-9B33-4BFB-BF58-AC2E40EF65D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{200FE63A-D738-4FB2-B688-2BBC55501AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="176">
   <si>
     <t>DERS KİTAPLARINDA YER ALAN KAREKOD BİLGİLERİ</t>
   </si>
@@ -517,6 +517,66 @@
   </si>
   <si>
     <t>mm_analitik43_mk</t>
+  </si>
+  <si>
+    <t>26.</t>
+  </si>
+  <si>
+    <t>27.</t>
+  </si>
+  <si>
+    <t>28.</t>
+  </si>
+  <si>
+    <t>29.</t>
+  </si>
+  <si>
+    <t>30.</t>
+  </si>
+  <si>
+    <t>Ana Karekod-2</t>
+  </si>
+  <si>
+    <t>mm_anakarekod2_mk</t>
+  </si>
+  <si>
+    <t>Ek Sorular 2.1</t>
+  </si>
+  <si>
+    <t>mm_eksorular21_mk</t>
+  </si>
+  <si>
+    <t>Ön Değerlendirme-21</t>
+  </si>
+  <si>
+    <t>mm_ondegerlendirme21_mk</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47958</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=53294</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=53295</t>
+  </si>
+  <si>
+    <t>Analitik-21</t>
+  </si>
+  <si>
+    <t>mm_analitik21_mk</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=53296</t>
+  </si>
+  <si>
+    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=57c6055c0a99d9273bf9838a0b9d9ba6&amp;resourceType=1&amp;resourceLocation=2</t>
+  </si>
+  <si>
+    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=a3d8ec681557effac25308ec06f30db8&amp;resourceType=1&amp;resourceLocation=2</t>
+  </si>
+  <si>
+    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=3abc4d5ce17e46fbdfedc0f0ee9d7dc2&amp;resourceType=1&amp;resourceLocation=2</t>
   </si>
 </sst>
 </file>
@@ -567,15 +627,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -635,25 +701,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -704,15 +757,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -728,10 +772,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Köprü" xfId="1" builtinId="8"/>
@@ -1013,48 +1060,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:F32"/>
+  <dimension ref="B2:F36"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="1.6640625" style="4" customWidth="1"/>
     <col min="2" max="2" width="4.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5546875" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.77734375" style="4" customWidth="1"/>
     <col min="6" max="6" width="117.5546875" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="8.77734375" style="4"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="23" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="25"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="22"/>
     </row>
     <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="23" t="s">
+      <c r="C4" s="19"/>
+      <c r="D4" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="5" spans="2:6" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>
@@ -1108,29 +1155,29 @@
       <c r="E8" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="11" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="11" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="10" t="s">
@@ -1147,7 +1194,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="10" t="s">
@@ -1164,7 +1211,7 @@
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="7" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="10" t="s">
@@ -1181,7 +1228,7 @@
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="10" t="s">
@@ -1198,7 +1245,7 @@
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="7" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="10" t="s">
@@ -1215,7 +1262,7 @@
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="7" t="s">
         <v>15</v>
       </c>
       <c r="C15" s="10" t="s">
@@ -1232,7 +1279,7 @@
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C16" s="10" t="s">
@@ -1249,7 +1296,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="7" t="s">
         <v>32</v>
       </c>
       <c r="C17" s="10" t="s">
@@ -1266,7 +1313,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="7" t="s">
         <v>33</v>
       </c>
       <c r="C18" s="10"/>
@@ -1275,213 +1322,282 @@
       <c r="F18" s="17"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="7" t="s">
         <v>34</v>
       </c>
       <c r="C19" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="F19" s="17"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="17"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D24" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="17"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="F24" s="17"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D25" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E25" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F25" s="11" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="10" t="s">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D26" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E26" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F26" s="11" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C22" s="10" t="s">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D27" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E27" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F27" s="25" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="8" t="s">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D28" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E28" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F28" s="11" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" s="8" t="s">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D29" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E29" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F29" s="11" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="8" t="s">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B30" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E30" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F30" s="11" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C26" s="10" t="s">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B31" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D31" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E31" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F31" s="11" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="C27" s="10" t="s">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B32" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C32" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D32" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E32" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="F32" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="C28" s="10" t="s">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B33" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D33" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E33" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="F28" s="11" t="s">
+      <c r="F33" s="11" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="C29" s="10" t="s">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B34" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D34" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="E29" s="26" t="s">
+      <c r="E34" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="F29" s="26" t="s">
+      <c r="F34" s="11" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="17"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="17"/>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B35" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="17"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B36" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1512,35 +1628,35 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="23" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="25"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="22"/>
     </row>
     <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="23" t="s">
+      <c r="C4" s="19"/>
+      <c r="D4" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="5" spans="2:6" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>

</xml_diff>

<commit_message>
AFTER GeoMATIK 3D v.0.1
</commit_message>
<xml_diff>
--- a/LİNKLER_Ademden.xlsx
+++ b/LİNKLER_Ademden.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mADEMatik\Desktop\GEO12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0C36BD-F907-400F-B909-D193B07708B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D41CBA3-BE2C-442A-8FC2-6FC6706D8EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="299">
   <si>
     <t>DERS KİTAPLARINDA YER ALAN KAREKOD BİLGİLERİ</t>
   </si>
@@ -922,6 +922,40 @@
   </si>
   <si>
     <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=d39726eda2de1a6e08effabf907c5490&amp;resourceType=1&amp;resourceLocation=2</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=46837</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47957</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47958</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47959</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47960</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47961</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47962</t>
+  </si>
+  <si>
+    <t>http://kitap.eba.gov.tr/KodSor.php?KOD=47963</t>
+  </si>
+  <si>
+    <t>25, 25, 31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34, 40, 42,
+48, 50, 53, 54, 57, 58, 63, 64, 72, 73, 75, 76, 79 </t>
+  </si>
+  <si>
+    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=2cb0002e70b3711dd473750d48e2cacd&amp;resourceType=1&amp;resourceLocation=2</t>
   </si>
 </sst>
 </file>
@@ -1233,7 +1267,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1413,18 +1447,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1434,6 +1462,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1475,6 +1509,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1763,9 +1803,9 @@
     <col min="1" max="1" width="1.6640625" style="4" customWidth="1"/>
     <col min="2" max="2" width="7.44140625" style="31" customWidth="1"/>
     <col min="3" max="3" width="6.44140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19" style="4" customWidth="1"/>
     <col min="5" max="5" width="23.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="21.21875" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="60" customWidth="1"/>
     <col min="8" max="8" width="100.6640625" style="60" customWidth="1"/>
     <col min="9" max="16384" width="8.77734375" style="4"/>
@@ -1836,7 +1876,7 @@
       <c r="G6" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="67" t="s">
+      <c r="H6" s="65" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1844,7 +1884,7 @@
       <c r="B7" s="73" t="s">
         <v>153</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="67" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="35">
@@ -1856,12 +1896,14 @@
       <c r="F7" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="G7" s="37"/>
+      <c r="G7" s="37" t="s">
+        <v>288</v>
+      </c>
       <c r="H7" s="38"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="74"/>
-      <c r="C8" s="65" t="s">
+      <c r="C8" s="63" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="20">
@@ -1882,7 +1924,7 @@
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="74"/>
-      <c r="C9" s="65" t="s">
+      <c r="C9" s="63" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="20">
@@ -1901,13 +1943,13 @@
         <v>263</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="74"/>
-      <c r="C10" s="65" t="s">
+      <c r="C10" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="23">
-        <v>34</v>
+      <c r="D10" s="23" t="s">
+        <v>297</v>
       </c>
       <c r="E10" s="22" t="s">
         <v>161</v>
@@ -1915,20 +1957,20 @@
       <c r="F10" s="22" t="s">
         <v>259</v>
       </c>
-      <c r="G10" s="58" t="s">
+      <c r="G10" s="82" t="s">
         <v>165</v>
       </c>
-      <c r="H10" s="39" t="s">
+      <c r="H10" s="83" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="74"/>
-      <c r="C11" s="65" t="s">
+      <c r="C11" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="20">
-        <v>25</v>
+      <c r="D11" s="20" t="s">
+        <v>296</v>
       </c>
       <c r="E11" s="22" t="s">
         <v>70</v>
@@ -1945,7 +1987,7 @@
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="74"/>
-      <c r="C12" s="65" t="s">
+      <c r="C12" s="63" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="20">
@@ -1966,7 +2008,7 @@
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="74"/>
-      <c r="C13" s="65" t="s">
+      <c r="C13" s="63" t="s">
         <v>13</v>
       </c>
       <c r="D13" s="20">
@@ -2000,7 +2042,7 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="74"/>
-      <c r="C15" s="65" t="s">
+      <c r="C15" s="63" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="20">
@@ -2021,7 +2063,7 @@
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" s="74"/>
-      <c r="C16" s="65" t="s">
+      <c r="C16" s="63" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="20">
@@ -2055,7 +2097,7 @@
     </row>
     <row r="18" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="75"/>
-      <c r="C18" s="66" t="s">
+      <c r="C18" s="64" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="40">
@@ -2086,7 +2128,7 @@
       <c r="B20" s="70" t="s">
         <v>154</v>
       </c>
-      <c r="C20" s="43" t="s">
+      <c r="C20" s="67" t="s">
         <v>1</v>
       </c>
       <c r="D20" s="43">
@@ -2098,12 +2140,14 @@
       <c r="F20" s="44" t="s">
         <v>115</v>
       </c>
-      <c r="G20" s="61"/>
+      <c r="G20" s="66" t="s">
+        <v>289</v>
+      </c>
       <c r="H20" s="45"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="71"/>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="63" t="s">
         <v>2</v>
       </c>
       <c r="D21" s="24">
@@ -2115,14 +2159,16 @@
       <c r="F21" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="G21" s="62" t="s">
+      <c r="G21" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="H21" s="46"/>
+      <c r="H21" s="47" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22" s="71"/>
-      <c r="C22" s="65" t="s">
+      <c r="C22" s="63" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="24">
@@ -2134,7 +2180,7 @@
       <c r="F22" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="G22" s="62" t="s">
+      <c r="G22" s="61" t="s">
         <v>175</v>
       </c>
       <c r="H22" s="47" t="s">
@@ -2149,7 +2195,7 @@
       <c r="D23" s="24"/>
       <c r="E23" s="24"/>
       <c r="F23" s="24"/>
-      <c r="G23" s="62" t="s">
+      <c r="G23" s="61" t="s">
         <v>176</v>
       </c>
       <c r="H23" s="47"/>
@@ -2162,7 +2208,7 @@
       <c r="D24" s="24"/>
       <c r="E24" s="24"/>
       <c r="F24" s="24"/>
-      <c r="G24" s="62" t="s">
+      <c r="G24" s="61" t="s">
         <v>177</v>
       </c>
       <c r="H24" s="47"/>
@@ -2175,7 +2221,7 @@
       <c r="D25" s="24"/>
       <c r="E25" s="24"/>
       <c r="F25" s="26"/>
-      <c r="G25" s="62" t="s">
+      <c r="G25" s="61" t="s">
         <v>178</v>
       </c>
       <c r="H25" s="47"/>
@@ -2188,7 +2234,7 @@
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
       <c r="F26" s="24"/>
-      <c r="G26" s="62" t="s">
+      <c r="G26" s="61" t="s">
         <v>179</v>
       </c>
       <c r="H26" s="47"/>
@@ -2201,14 +2247,14 @@
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
       <c r="F27" s="24"/>
-      <c r="G27" s="62" t="s">
+      <c r="G27" s="61" t="s">
         <v>180</v>
       </c>
       <c r="H27" s="47"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B28" s="71"/>
-      <c r="C28" s="65" t="s">
+      <c r="C28" s="63" t="s">
         <v>15</v>
       </c>
       <c r="D28" s="24">
@@ -2220,7 +2266,7 @@
       <c r="F28" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="G28" s="62" t="s">
+      <c r="G28" s="61" t="s">
         <v>181</v>
       </c>
       <c r="H28" s="47" t="s">
@@ -2235,7 +2281,7 @@
       <c r="D29" s="24"/>
       <c r="E29" s="24"/>
       <c r="F29" s="26"/>
-      <c r="G29" s="62" t="s">
+      <c r="G29" s="61" t="s">
         <v>182</v>
       </c>
       <c r="H29" s="47"/>
@@ -2248,14 +2294,14 @@
       <c r="D30" s="24"/>
       <c r="E30" s="24"/>
       <c r="F30" s="26"/>
-      <c r="G30" s="62" t="s">
+      <c r="G30" s="61" t="s">
         <v>183</v>
       </c>
       <c r="H30" s="47"/>
     </row>
     <row r="31" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="72"/>
-      <c r="C31" s="66" t="s">
+      <c r="C31" s="64" t="s">
         <v>19</v>
       </c>
       <c r="D31" s="48">
@@ -2267,7 +2313,7 @@
       <c r="F31" s="49" t="s">
         <v>119</v>
       </c>
-      <c r="G31" s="63" t="s">
+      <c r="G31" s="62" t="s">
         <v>184</v>
       </c>
       <c r="H31" s="50" t="s">
@@ -2298,12 +2344,14 @@
       <c r="F33" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="G33" s="64"/>
+      <c r="G33" s="37" t="s">
+        <v>290</v>
+      </c>
       <c r="H33" s="51"/>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B34" s="74"/>
-      <c r="C34" s="65" t="s">
+      <c r="C34" s="63" t="s">
         <v>2</v>
       </c>
       <c r="D34" s="20">
@@ -2324,7 +2372,7 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B35" s="74"/>
-      <c r="C35" s="65" t="s">
+      <c r="C35" s="63" t="s">
         <v>9</v>
       </c>
       <c r="D35" s="20">
@@ -2410,7 +2458,7 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B41" s="74"/>
-      <c r="C41" s="65" t="s">
+      <c r="C41" s="63" t="s">
         <v>15</v>
       </c>
       <c r="D41" s="20">
@@ -2457,7 +2505,7 @@
     </row>
     <row r="44" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="75"/>
-      <c r="C44" s="66" t="s">
+      <c r="C44" s="64" t="s">
         <v>19</v>
       </c>
       <c r="D44" s="40">
@@ -2500,7 +2548,9 @@
       <c r="F46" s="53" t="s">
         <v>125</v>
       </c>
-      <c r="G46" s="61"/>
+      <c r="G46" s="66" t="s">
+        <v>291</v>
+      </c>
       <c r="H46" s="45"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
@@ -2517,7 +2567,7 @@
       <c r="F47" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="G47" s="62" t="s">
+      <c r="G47" s="61" t="s">
         <v>196</v>
       </c>
       <c r="H47" s="46"/>
@@ -2536,7 +2586,7 @@
       <c r="F48" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="G48" s="62" t="s">
+      <c r="G48" s="61" t="s">
         <v>197</v>
       </c>
       <c r="H48" s="46"/>
@@ -2555,7 +2605,7 @@
       <c r="F49" s="26" t="s">
         <v>260</v>
       </c>
-      <c r="G49" s="62" t="s">
+      <c r="G49" s="61" t="s">
         <v>198</v>
       </c>
       <c r="H49" s="47" t="s">
@@ -2570,7 +2620,7 @@
       <c r="D50" s="24"/>
       <c r="E50" s="24"/>
       <c r="F50" s="24"/>
-      <c r="G50" s="62" t="s">
+      <c r="G50" s="61" t="s">
         <v>199</v>
       </c>
       <c r="H50" s="46"/>
@@ -2583,7 +2633,7 @@
       <c r="D51" s="24"/>
       <c r="E51" s="24"/>
       <c r="F51" s="26"/>
-      <c r="G51" s="62" t="s">
+      <c r="G51" s="61" t="s">
         <v>200</v>
       </c>
       <c r="H51" s="46"/>
@@ -2596,7 +2646,7 @@
       <c r="D52" s="24"/>
       <c r="E52" s="24"/>
       <c r="F52" s="26"/>
-      <c r="G52" s="62" t="s">
+      <c r="G52" s="61" t="s">
         <v>201</v>
       </c>
       <c r="H52" s="46"/>
@@ -2609,7 +2659,7 @@
       <c r="D53" s="24"/>
       <c r="E53" s="24"/>
       <c r="F53" s="24"/>
-      <c r="G53" s="62" t="s">
+      <c r="G53" s="61" t="s">
         <v>202</v>
       </c>
       <c r="H53" s="46"/>
@@ -2628,7 +2678,7 @@
       <c r="F54" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="G54" s="62" t="s">
+      <c r="G54" s="61" t="s">
         <v>203</v>
       </c>
       <c r="H54" s="46"/>
@@ -2641,7 +2691,7 @@
       <c r="D55" s="24"/>
       <c r="E55" s="24"/>
       <c r="F55" s="26"/>
-      <c r="G55" s="62" t="s">
+      <c r="G55" s="61" t="s">
         <v>204</v>
       </c>
       <c r="H55" s="46"/>
@@ -2654,7 +2704,7 @@
       <c r="D56" s="24"/>
       <c r="E56" s="24"/>
       <c r="F56" s="26"/>
-      <c r="G56" s="62" t="s">
+      <c r="G56" s="61" t="s">
         <v>205</v>
       </c>
       <c r="H56" s="46"/>
@@ -2673,7 +2723,7 @@
       <c r="F57" s="49" t="s">
         <v>129</v>
       </c>
-      <c r="G57" s="63" t="s">
+      <c r="G57" s="62" t="s">
         <v>206</v>
       </c>
       <c r="H57" s="54"/>
@@ -2702,7 +2752,9 @@
       <c r="F59" s="36" t="s">
         <v>130</v>
       </c>
-      <c r="G59" s="64"/>
+      <c r="G59" s="37" t="s">
+        <v>292</v>
+      </c>
       <c r="H59" s="51"/>
     </row>
     <row r="60" spans="2:8" x14ac:dyDescent="0.3">
@@ -2726,7 +2778,7 @@
     </row>
     <row r="61" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B61" s="74"/>
-      <c r="C61" s="65" t="s">
+      <c r="C61" s="63" t="s">
         <v>9</v>
       </c>
       <c r="D61" s="20">
@@ -2812,7 +2864,7 @@
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B67" s="74"/>
-      <c r="C67" s="65" t="s">
+      <c r="C67" s="63" t="s">
         <v>15</v>
       </c>
       <c r="D67" s="20">
@@ -2859,7 +2911,7 @@
     </row>
     <row r="70" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B70" s="75"/>
-      <c r="C70" s="66" t="s">
+      <c r="C70" s="64" t="s">
         <v>19</v>
       </c>
       <c r="D70" s="40">
@@ -2902,7 +2954,9 @@
       <c r="F72" s="53" t="s">
         <v>135</v>
       </c>
-      <c r="G72" s="61"/>
+      <c r="G72" s="66" t="s">
+        <v>293</v>
+      </c>
       <c r="H72" s="45"/>
     </row>
     <row r="73" spans="2:8" x14ac:dyDescent="0.3">
@@ -2919,14 +2973,14 @@
       <c r="F73" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="G73" s="62" t="s">
+      <c r="G73" s="61" t="s">
         <v>218</v>
       </c>
       <c r="H73" s="46"/>
     </row>
     <row r="74" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B74" s="71"/>
-      <c r="C74" s="65" t="s">
+      <c r="C74" s="63" t="s">
         <v>9</v>
       </c>
       <c r="D74" s="24">
@@ -2938,7 +2992,7 @@
       <c r="F74" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="G74" s="62" t="s">
+      <c r="G74" s="61" t="s">
         <v>219</v>
       </c>
       <c r="H74" s="47" t="s">
@@ -2947,7 +3001,7 @@
     </row>
     <row r="75" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B75" s="71"/>
-      <c r="C75" s="65" t="s">
+      <c r="C75" s="63" t="s">
         <v>10</v>
       </c>
       <c r="D75" s="24">
@@ -2959,7 +3013,7 @@
       <c r="F75" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="G75" s="62" t="s">
+      <c r="G75" s="61" t="s">
         <v>220</v>
       </c>
       <c r="H75" s="47" t="s">
@@ -2974,7 +3028,7 @@
       <c r="D76" s="24"/>
       <c r="E76" s="24"/>
       <c r="F76" s="24"/>
-      <c r="G76" s="62" t="s">
+      <c r="G76" s="61" t="s">
         <v>221</v>
       </c>
       <c r="H76" s="46"/>
@@ -2987,7 +3041,7 @@
       <c r="D77" s="24"/>
       <c r="E77" s="24"/>
       <c r="F77" s="24"/>
-      <c r="G77" s="62" t="s">
+      <c r="G77" s="61" t="s">
         <v>222</v>
       </c>
       <c r="H77" s="46"/>
@@ -3000,7 +3054,7 @@
       <c r="D78" s="24"/>
       <c r="E78" s="24"/>
       <c r="F78" s="26"/>
-      <c r="G78" s="62" t="s">
+      <c r="G78" s="61" t="s">
         <v>223</v>
       </c>
       <c r="H78" s="46"/>
@@ -3013,14 +3067,14 @@
       <c r="D79" s="24"/>
       <c r="E79" s="24"/>
       <c r="F79" s="24"/>
-      <c r="G79" s="62" t="s">
+      <c r="G79" s="61" t="s">
         <v>224</v>
       </c>
       <c r="H79" s="46"/>
     </row>
     <row r="80" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B80" s="71"/>
-      <c r="C80" s="65" t="s">
+      <c r="C80" s="63" t="s">
         <v>15</v>
       </c>
       <c r="D80" s="24">
@@ -3032,7 +3086,7 @@
       <c r="F80" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="G80" s="62" t="s">
+      <c r="G80" s="61" t="s">
         <v>225</v>
       </c>
       <c r="H80" s="47" t="s">
@@ -3047,7 +3101,7 @@
       <c r="D81" s="24"/>
       <c r="E81" s="24"/>
       <c r="F81" s="26"/>
-      <c r="G81" s="62" t="s">
+      <c r="G81" s="61" t="s">
         <v>226</v>
       </c>
       <c r="H81" s="46"/>
@@ -3060,14 +3114,14 @@
       <c r="D82" s="24"/>
       <c r="E82" s="24"/>
       <c r="F82" s="26"/>
-      <c r="G82" s="62" t="s">
+      <c r="G82" s="61" t="s">
         <v>227</v>
       </c>
       <c r="H82" s="46"/>
     </row>
     <row r="83" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B83" s="72"/>
-      <c r="C83" s="66" t="s">
+      <c r="C83" s="64" t="s">
         <v>19</v>
       </c>
       <c r="D83" s="48">
@@ -3079,7 +3133,7 @@
       <c r="F83" s="49" t="s">
         <v>140</v>
       </c>
-      <c r="G83" s="63" t="s">
+      <c r="G83" s="62" t="s">
         <v>228</v>
       </c>
       <c r="H83" s="50" t="s">
@@ -3110,7 +3164,9 @@
       <c r="F85" s="36" t="s">
         <v>141</v>
       </c>
-      <c r="G85" s="64"/>
+      <c r="G85" s="37" t="s">
+        <v>294</v>
+      </c>
       <c r="H85" s="51"/>
     </row>
     <row r="86" spans="2:8" x14ac:dyDescent="0.3">
@@ -3134,7 +3190,7 @@
     </row>
     <row r="87" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B87" s="74"/>
-      <c r="C87" s="65" t="s">
+      <c r="C87" s="63" t="s">
         <v>9</v>
       </c>
       <c r="D87" s="20">
@@ -3220,7 +3276,7 @@
     </row>
     <row r="93" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B93" s="74"/>
-      <c r="C93" s="65" t="s">
+      <c r="C93" s="63" t="s">
         <v>15</v>
       </c>
       <c r="D93" s="20" t="s">
@@ -3267,7 +3323,7 @@
     </row>
     <row r="96" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B96" s="75"/>
-      <c r="C96" s="66" t="s">
+      <c r="C96" s="64" t="s">
         <v>19</v>
       </c>
       <c r="D96" s="40">
@@ -3310,7 +3366,9 @@
       <c r="F98" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="G98" s="61"/>
+      <c r="G98" s="66" t="s">
+        <v>295</v>
+      </c>
       <c r="H98" s="55"/>
     </row>
     <row r="99" spans="2:8" x14ac:dyDescent="0.3">
@@ -3327,7 +3385,7 @@
       <c r="F99" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="G99" s="62" t="s">
+      <c r="G99" s="61" t="s">
         <v>240</v>
       </c>
       <c r="H99" s="47"/>
@@ -3346,7 +3404,7 @@
       <c r="F100" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G100" s="62" t="s">
+      <c r="G100" s="61" t="s">
         <v>241</v>
       </c>
       <c r="H100" s="47"/>
@@ -3359,7 +3417,7 @@
       <c r="D101" s="24"/>
       <c r="E101" s="24"/>
       <c r="F101" s="24"/>
-      <c r="G101" s="62" t="s">
+      <c r="G101" s="61" t="s">
         <v>242</v>
       </c>
       <c r="H101" s="47"/>
@@ -3372,7 +3430,7 @@
       <c r="D102" s="24"/>
       <c r="E102" s="24"/>
       <c r="F102" s="24"/>
-      <c r="G102" s="62" t="s">
+      <c r="G102" s="61" t="s">
         <v>243</v>
       </c>
       <c r="H102" s="47"/>
@@ -3385,7 +3443,7 @@
       <c r="D103" s="24"/>
       <c r="E103" s="24"/>
       <c r="F103" s="26"/>
-      <c r="G103" s="62" t="s">
+      <c r="G103" s="61" t="s">
         <v>244</v>
       </c>
       <c r="H103" s="47"/>
@@ -3398,7 +3456,7 @@
       <c r="D104" s="24"/>
       <c r="E104" s="24"/>
       <c r="F104" s="26"/>
-      <c r="G104" s="62" t="s">
+      <c r="G104" s="61" t="s">
         <v>245</v>
       </c>
       <c r="H104" s="47"/>
@@ -3411,7 +3469,7 @@
       <c r="D105" s="24"/>
       <c r="E105" s="24"/>
       <c r="F105" s="24"/>
-      <c r="G105" s="62" t="s">
+      <c r="G105" s="61" t="s">
         <v>246</v>
       </c>
       <c r="H105" s="47"/>
@@ -3430,7 +3488,7 @@
       <c r="F106" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="G106" s="62" t="s">
+      <c r="G106" s="61" t="s">
         <v>247</v>
       </c>
       <c r="H106" s="47"/>
@@ -3443,7 +3501,7 @@
       <c r="D107" s="24"/>
       <c r="E107" s="24"/>
       <c r="F107" s="26"/>
-      <c r="G107" s="62" t="s">
+      <c r="G107" s="61" t="s">
         <v>248</v>
       </c>
       <c r="H107" s="47"/>
@@ -3456,7 +3514,7 @@
       <c r="D108" s="24"/>
       <c r="E108" s="24"/>
       <c r="F108" s="26"/>
-      <c r="G108" s="62" t="s">
+      <c r="G108" s="61" t="s">
         <v>249</v>
       </c>
       <c r="H108" s="47"/>
@@ -3475,7 +3533,7 @@
       <c r="F109" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="G109" s="63" t="s">
+      <c r="G109" s="62" t="s">
         <v>250</v>
       </c>
       <c r="H109" s="54"/>

</xml_diff>

<commit_message>
AFTER AVCELL EDIT ARROWS
</commit_message>
<xml_diff>
--- a/LİNKLER_Ademden.xlsx
+++ b/LİNKLER_Ademden.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mADEMatik\Desktop\GEO12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BA29E5-AD45-434B-8B32-32DDB01B9D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A22AF26E-1BF2-4866-812C-8D65A5A00E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="319">
   <si>
     <t>DERS KİTAPLARINDA YER ALAN KAREKOD BİLGİLERİ</t>
   </si>
@@ -993,6 +993,27 @@
     <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=0e5aa0333fdcff9dff7e9dec4b39269a&amp;resourceType=1&amp;resourceLocation=2</t>
   </si>
   <si>
+    <t>Akran 8.1</t>
+  </si>
+  <si>
+    <t>mm_81akran_mk</t>
+  </si>
+  <si>
+    <t>Grup 8.1</t>
+  </si>
+  <si>
+    <t>mm_81grup_mk</t>
+  </si>
+  <si>
+    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=ad2bcdbe346be64237f6399eb85e4300&amp;resourceType=1&amp;resourceLocation=2</t>
+  </si>
+  <si>
+    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=075d0be38ae0e1bcf74c3aa830d29e1e&amp;resourceType=1&amp;resourceLocation=2</t>
+  </si>
+  <si>
+    <t>385, 390, 394, 396</t>
+  </si>
+  <si>
     <t>T1: 34, 40, 42
 T2: 48, 52, 56, 57, 59, 60, 61, 63, 64, 66, 67, 72, 73, 74, 76, 83
 T3: 99, 100, 101, 107, 112, 115
@@ -1000,25 +1021,7 @@
 T5: 165, 170, 177, 179, 181, 193
 T6: 248, 254, 256, 284, 285, 294, 300, 303
 T7:
-T8:</t>
-  </si>
-  <si>
-    <t>Akran 8.1</t>
-  </si>
-  <si>
-    <t>mm_81akran_mk</t>
-  </si>
-  <si>
-    <t>Grup 8.1</t>
-  </si>
-  <si>
-    <t>mm_81grup_mk</t>
-  </si>
-  <si>
-    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=ad2bcdbe346be64237f6399eb85e4300&amp;resourceType=1&amp;resourceLocation=2</t>
-  </si>
-  <si>
-    <t>https://ders.eba.gov.tr/ders//redirectContent.jsp?resourceId=075d0be38ae0e1bcf74c3aa830d29e1e&amp;resourceType=1&amp;resourceLocation=2</t>
+T8: -</t>
   </si>
 </sst>
 </file>
@@ -1077,7 +1080,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1096,12 +1099,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="19">
     <border>
@@ -1372,7 +1369,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1519,18 +1516,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -1545,9 +1533,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1914,41 +1899,41 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="72" t="s">
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
     </row>
     <row r="4" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="71"/>
-      <c r="D4" s="71"/>
-      <c r="E4" s="71"/>
-      <c r="F4" s="72" t="s">
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="72"/>
-      <c r="H4" s="72"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
     </row>
     <row r="5" spans="2:8" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="21"/>
@@ -1960,52 +1945,52 @@
       <c r="H5" s="44"/>
     </row>
     <row r="6" spans="2:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="60" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="61" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="65" t="s">
+      <c r="D6" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="E6" s="66" t="s">
+      <c r="E6" s="62" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="65" t="s">
+      <c r="F6" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="67" t="s">
+      <c r="G6" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="68" t="s">
+      <c r="H6" s="64" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B7" s="79" t="s">
+      <c r="B7" s="75" t="s">
         <v>153</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="60">
+      <c r="D7" s="56">
         <v>13</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="57" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="57" t="s">
         <v>106</v>
       </c>
-      <c r="G7" s="62" t="s">
+      <c r="G7" s="58" t="s">
         <v>284</v>
       </c>
-      <c r="H7" s="63"/>
+      <c r="H7" s="59"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="77"/>
-      <c r="C8" s="50" t="s">
+      <c r="B8" s="73"/>
+      <c r="C8" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="15">
@@ -2025,8 +2010,8 @@
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="77"/>
-      <c r="C9" s="50" t="s">
+      <c r="B9" s="73"/>
+      <c r="C9" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="15">
@@ -2046,12 +2031,12 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="77"/>
-      <c r="C10" s="50" t="s">
+      <c r="B10" s="73"/>
+      <c r="C10" s="15" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>306</v>
@@ -2059,16 +2044,16 @@
       <c r="F10" s="17" t="s">
         <v>257</v>
       </c>
-      <c r="G10" s="54" t="s">
+      <c r="G10" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="H10" s="55" t="s">
+      <c r="H10" s="52" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="77"/>
-      <c r="C11" s="50" t="s">
+      <c r="B11" s="73"/>
+      <c r="C11" s="15" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="15" t="s">
@@ -2088,8 +2073,8 @@
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="77"/>
-      <c r="C12" s="50" t="s">
+      <c r="B12" s="73"/>
+      <c r="C12" s="15" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="15">
@@ -2109,8 +2094,8 @@
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="77"/>
-      <c r="C13" s="50" t="s">
+      <c r="B13" s="73"/>
+      <c r="C13" s="15" t="s">
         <v>13</v>
       </c>
       <c r="D13" s="15">
@@ -2130,7 +2115,7 @@
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="77"/>
+      <c r="B14" s="73"/>
       <c r="C14" s="15" t="s">
         <v>14</v>
       </c>
@@ -2143,8 +2128,8 @@
       <c r="H14" s="28"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="77"/>
-      <c r="C15" s="50" t="s">
+      <c r="B15" s="73"/>
+      <c r="C15" s="15" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="15">
@@ -2164,8 +2149,8 @@
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="77"/>
-      <c r="C16" s="50" t="s">
+      <c r="B16" s="73"/>
+      <c r="C16" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="15">
@@ -2185,7 +2170,7 @@
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B17" s="77"/>
+      <c r="B17" s="73"/>
       <c r="C17" s="15" t="s">
         <v>18</v>
       </c>
@@ -2198,8 +2183,8 @@
       <c r="H17" s="28"/>
     </row>
     <row r="18" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="78"/>
-      <c r="C18" s="51" t="s">
+      <c r="B18" s="74"/>
+      <c r="C18" s="29" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="29">
@@ -2220,10 +2205,10 @@
     </row>
     <row r="19" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B20" s="73" t="s">
+      <c r="B20" s="69" t="s">
         <v>154</v>
       </c>
-      <c r="C20" s="53" t="s">
+      <c r="C20" s="32" t="s">
         <v>1</v>
       </c>
       <c r="D20" s="32">
@@ -2235,14 +2220,14 @@
       <c r="F20" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="G20" s="52" t="s">
+      <c r="G20" s="50" t="s">
         <v>285</v>
       </c>
       <c r="H20" s="34"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B21" s="74"/>
-      <c r="C21" s="50" t="s">
+      <c r="B21" s="70"/>
+      <c r="C21" s="18" t="s">
         <v>2</v>
       </c>
       <c r="D21" s="18">
@@ -2262,8 +2247,8 @@
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="74"/>
-      <c r="C22" s="50" t="s">
+      <c r="B22" s="70"/>
+      <c r="C22" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="18">
@@ -2283,7 +2268,7 @@
       </c>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B23" s="74"/>
+      <c r="B23" s="70"/>
       <c r="C23" s="18" t="s">
         <v>10</v>
       </c>
@@ -2296,7 +2281,7 @@
       <c r="H23" s="36"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B24" s="74"/>
+      <c r="B24" s="70"/>
       <c r="C24" s="18" t="s">
         <v>11</v>
       </c>
@@ -2309,7 +2294,7 @@
       <c r="H24" s="36"/>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B25" s="74"/>
+      <c r="B25" s="70"/>
       <c r="C25" s="18" t="s">
         <v>12</v>
       </c>
@@ -2322,7 +2307,7 @@
       <c r="H25" s="36"/>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B26" s="74"/>
+      <c r="B26" s="70"/>
       <c r="C26" s="18" t="s">
         <v>13</v>
       </c>
@@ -2335,7 +2320,7 @@
       <c r="H26" s="36"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B27" s="74"/>
+      <c r="B27" s="70"/>
       <c r="C27" s="18" t="s">
         <v>14</v>
       </c>
@@ -2348,8 +2333,8 @@
       <c r="H27" s="36"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B28" s="74"/>
-      <c r="C28" s="50" t="s">
+      <c r="B28" s="70"/>
+      <c r="C28" s="18" t="s">
         <v>15</v>
       </c>
       <c r="D28" s="18">
@@ -2369,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B29" s="74"/>
+      <c r="B29" s="70"/>
       <c r="C29" s="18" t="s">
         <v>16</v>
       </c>
@@ -2382,7 +2367,7 @@
       <c r="H29" s="36"/>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B30" s="74"/>
+      <c r="B30" s="70"/>
       <c r="C30" s="18" t="s">
         <v>18</v>
       </c>
@@ -2395,8 +2380,8 @@
       <c r="H30" s="36"/>
     </row>
     <row r="31" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="75"/>
-      <c r="C31" s="51" t="s">
+      <c r="B31" s="71"/>
+      <c r="C31" s="37" t="s">
         <v>19</v>
       </c>
       <c r="D31" s="37">
@@ -2417,10 +2402,10 @@
     </row>
     <row r="32" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F32" s="24"/>
-      <c r="H32" s="56"/>
+      <c r="H32" s="53"/>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B33" s="76" t="s">
+      <c r="B33" s="72" t="s">
         <v>155</v>
       </c>
       <c r="C33" s="25" t="s">
@@ -2441,7 +2426,7 @@
       <c r="H33" s="40"/>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B34" s="77"/>
+      <c r="B34" s="73"/>
       <c r="C34" s="15" t="s">
         <v>2</v>
       </c>
@@ -2462,7 +2447,7 @@
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B35" s="77"/>
+      <c r="B35" s="73"/>
       <c r="C35" s="15" t="s">
         <v>9</v>
       </c>
@@ -2483,7 +2468,7 @@
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B36" s="77"/>
+      <c r="B36" s="73"/>
       <c r="C36" s="15" t="s">
         <v>10</v>
       </c>
@@ -2496,7 +2481,7 @@
       <c r="H36" s="28"/>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B37" s="77"/>
+      <c r="B37" s="73"/>
       <c r="C37" s="15" t="s">
         <v>11</v>
       </c>
@@ -2509,7 +2494,7 @@
       <c r="H37" s="41"/>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B38" s="77"/>
+      <c r="B38" s="73"/>
       <c r="C38" s="15" t="s">
         <v>12</v>
       </c>
@@ -2522,7 +2507,7 @@
       <c r="H38" s="41"/>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B39" s="77"/>
+      <c r="B39" s="73"/>
       <c r="C39" s="15" t="s">
         <v>13</v>
       </c>
@@ -2535,7 +2520,7 @@
       <c r="H39" s="41"/>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B40" s="77"/>
+      <c r="B40" s="73"/>
       <c r="C40" s="15" t="s">
         <v>14</v>
       </c>
@@ -2548,7 +2533,7 @@
       <c r="H40" s="41"/>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B41" s="77"/>
+      <c r="B41" s="73"/>
       <c r="C41" s="15" t="s">
         <v>15</v>
       </c>
@@ -2569,7 +2554,7 @@
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B42" s="77"/>
+      <c r="B42" s="73"/>
       <c r="C42" s="15" t="s">
         <v>16</v>
       </c>
@@ -2582,7 +2567,7 @@
       <c r="H42" s="41"/>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B43" s="77"/>
+      <c r="B43" s="73"/>
       <c r="C43" s="15" t="s">
         <v>18</v>
       </c>
@@ -2595,7 +2580,7 @@
       <c r="H43" s="41"/>
     </row>
     <row r="44" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="78"/>
+      <c r="B44" s="74"/>
       <c r="C44" s="29" t="s">
         <v>19</v>
       </c>
@@ -2617,10 +2602,10 @@
     </row>
     <row r="45" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F45" s="24"/>
-      <c r="H45" s="57"/>
+      <c r="H45" s="54"/>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B46" s="73" t="s">
+      <c r="B46" s="69" t="s">
         <v>156</v>
       </c>
       <c r="C46" s="32" t="s">
@@ -2635,13 +2620,13 @@
       <c r="F46" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="G46" s="52" t="s">
+      <c r="G46" s="50" t="s">
         <v>287</v>
       </c>
       <c r="H46" s="34"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B47" s="74"/>
+      <c r="B47" s="70"/>
       <c r="C47" s="18" t="s">
         <v>2</v>
       </c>
@@ -2662,7 +2647,7 @@
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B48" s="74"/>
+      <c r="B48" s="70"/>
       <c r="C48" s="18" t="s">
         <v>9</v>
       </c>
@@ -2683,7 +2668,7 @@
       </c>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B49" s="74"/>
+      <c r="B49" s="70"/>
       <c r="C49" s="18" t="s">
         <v>10</v>
       </c>
@@ -2704,7 +2689,7 @@
       </c>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B50" s="74"/>
+      <c r="B50" s="70"/>
       <c r="C50" s="18" t="s">
         <v>11</v>
       </c>
@@ -2717,7 +2702,7 @@
       <c r="H50" s="35"/>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B51" s="74"/>
+      <c r="B51" s="70"/>
       <c r="C51" s="18" t="s">
         <v>12</v>
       </c>
@@ -2730,7 +2715,7 @@
       <c r="H51" s="35"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B52" s="74"/>
+      <c r="B52" s="70"/>
       <c r="C52" s="18" t="s">
         <v>13</v>
       </c>
@@ -2743,7 +2728,7 @@
       <c r="H52" s="35"/>
     </row>
     <row r="53" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B53" s="74"/>
+      <c r="B53" s="70"/>
       <c r="C53" s="18" t="s">
         <v>14</v>
       </c>
@@ -2756,7 +2741,7 @@
       <c r="H53" s="35"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B54" s="74"/>
+      <c r="B54" s="70"/>
       <c r="C54" s="18" t="s">
         <v>15</v>
       </c>
@@ -2777,7 +2762,7 @@
       </c>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B55" s="74"/>
+      <c r="B55" s="70"/>
       <c r="C55" s="18" t="s">
         <v>16</v>
       </c>
@@ -2790,7 +2775,7 @@
       <c r="H55" s="35"/>
     </row>
     <row r="56" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B56" s="74"/>
+      <c r="B56" s="70"/>
       <c r="C56" s="18" t="s">
         <v>18</v>
       </c>
@@ -2803,7 +2788,7 @@
       <c r="H56" s="35"/>
     </row>
     <row r="57" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B57" s="75"/>
+      <c r="B57" s="71"/>
       <c r="C57" s="37" t="s">
         <v>19</v>
       </c>
@@ -2825,10 +2810,10 @@
     </row>
     <row r="58" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F58" s="24"/>
-      <c r="H58" s="58"/>
+      <c r="H58" s="55"/>
     </row>
     <row r="59" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B59" s="76" t="s">
+      <c r="B59" s="72" t="s">
         <v>157</v>
       </c>
       <c r="C59" s="25" t="s">
@@ -2849,7 +2834,7 @@
       <c r="H59" s="40"/>
     </row>
     <row r="60" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B60" s="77"/>
+      <c r="B60" s="73"/>
       <c r="C60" s="15" t="s">
         <v>2</v>
       </c>
@@ -2870,7 +2855,7 @@
       </c>
     </row>
     <row r="61" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B61" s="77"/>
+      <c r="B61" s="73"/>
       <c r="C61" s="15" t="s">
         <v>9</v>
       </c>
@@ -2891,7 +2876,7 @@
       </c>
     </row>
     <row r="62" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B62" s="77"/>
+      <c r="B62" s="73"/>
       <c r="C62" s="15" t="s">
         <v>10</v>
       </c>
@@ -2904,7 +2889,7 @@
       <c r="H62" s="41"/>
     </row>
     <row r="63" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B63" s="77"/>
+      <c r="B63" s="73"/>
       <c r="C63" s="15" t="s">
         <v>11</v>
       </c>
@@ -2917,7 +2902,7 @@
       <c r="H63" s="41"/>
     </row>
     <row r="64" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B64" s="77"/>
+      <c r="B64" s="73"/>
       <c r="C64" s="15" t="s">
         <v>12</v>
       </c>
@@ -2930,7 +2915,7 @@
       <c r="H64" s="41"/>
     </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B65" s="77"/>
+      <c r="B65" s="73"/>
       <c r="C65" s="15" t="s">
         <v>13</v>
       </c>
@@ -2943,7 +2928,7 @@
       <c r="H65" s="41"/>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B66" s="77"/>
+      <c r="B66" s="73"/>
       <c r="C66" s="15" t="s">
         <v>14</v>
       </c>
@@ -2956,7 +2941,7 @@
       <c r="H66" s="41"/>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B67" s="77"/>
+      <c r="B67" s="73"/>
       <c r="C67" s="15" t="s">
         <v>15</v>
       </c>
@@ -2977,7 +2962,7 @@
       </c>
     </row>
     <row r="68" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B68" s="77"/>
+      <c r="B68" s="73"/>
       <c r="C68" s="15" t="s">
         <v>16</v>
       </c>
@@ -2990,7 +2975,7 @@
       <c r="H68" s="41"/>
     </row>
     <row r="69" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B69" s="77"/>
+      <c r="B69" s="73"/>
       <c r="C69" s="15" t="s">
         <v>18</v>
       </c>
@@ -3003,7 +2988,7 @@
       <c r="H69" s="41"/>
     </row>
     <row r="70" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B70" s="78"/>
+      <c r="B70" s="74"/>
       <c r="C70" s="29" t="s">
         <v>19</v>
       </c>
@@ -3016,7 +3001,7 @@
       <c r="F70" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="G70" s="69" t="s">
+      <c r="G70" s="65" t="s">
         <v>215</v>
       </c>
       <c r="H70" s="31" t="s">
@@ -3025,13 +3010,13 @@
     </row>
     <row r="71" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F71" s="24"/>
-      <c r="H71" s="58"/>
+      <c r="H71" s="55"/>
     </row>
     <row r="72" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B72" s="73" t="s">
+      <c r="B72" s="69" t="s">
         <v>158</v>
       </c>
-      <c r="C72" s="53" t="s">
+      <c r="C72" s="32" t="s">
         <v>1</v>
       </c>
       <c r="D72" s="32">
@@ -3043,14 +3028,14 @@
       <c r="F72" s="42" t="s">
         <v>135</v>
       </c>
-      <c r="G72" s="52" t="s">
+      <c r="G72" s="50" t="s">
         <v>289</v>
       </c>
       <c r="H72" s="34"/>
     </row>
     <row r="73" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B73" s="74"/>
-      <c r="C73" s="50" t="s">
+      <c r="B73" s="70"/>
+      <c r="C73" s="18" t="s">
         <v>2</v>
       </c>
       <c r="D73" s="18">
@@ -3070,8 +3055,8 @@
       </c>
     </row>
     <row r="74" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B74" s="74"/>
-      <c r="C74" s="50" t="s">
+      <c r="B74" s="70"/>
+      <c r="C74" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D74" s="18">
@@ -3091,7 +3076,7 @@
       </c>
     </row>
     <row r="75" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B75" s="74"/>
+      <c r="B75" s="70"/>
       <c r="C75" s="18" t="s">
         <v>10</v>
       </c>
@@ -3110,7 +3095,7 @@
       </c>
     </row>
     <row r="76" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B76" s="74"/>
+      <c r="B76" s="70"/>
       <c r="C76" s="18" t="s">
         <v>11</v>
       </c>
@@ -3123,7 +3108,7 @@
       <c r="H76" s="35"/>
     </row>
     <row r="77" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B77" s="74"/>
+      <c r="B77" s="70"/>
       <c r="C77" s="18" t="s">
         <v>12</v>
       </c>
@@ -3136,7 +3121,7 @@
       <c r="H77" s="35"/>
     </row>
     <row r="78" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B78" s="74"/>
+      <c r="B78" s="70"/>
       <c r="C78" s="18" t="s">
         <v>13</v>
       </c>
@@ -3149,7 +3134,7 @@
       <c r="H78" s="35"/>
     </row>
     <row r="79" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B79" s="74"/>
+      <c r="B79" s="70"/>
       <c r="C79" s="18" t="s">
         <v>14</v>
       </c>
@@ -3162,8 +3147,8 @@
       <c r="H79" s="35"/>
     </row>
     <row r="80" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B80" s="74"/>
-      <c r="C80" s="50" t="s">
+      <c r="B80" s="70"/>
+      <c r="C80" s="18" t="s">
         <v>15</v>
       </c>
       <c r="D80" s="18">
@@ -3183,7 +3168,7 @@
       </c>
     </row>
     <row r="81" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B81" s="74"/>
+      <c r="B81" s="70"/>
       <c r="C81" s="18" t="s">
         <v>16</v>
       </c>
@@ -3196,7 +3181,7 @@
       <c r="H81" s="35"/>
     </row>
     <row r="82" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B82" s="74"/>
+      <c r="B82" s="70"/>
       <c r="C82" s="18" t="s">
         <v>18</v>
       </c>
@@ -3209,8 +3194,8 @@
       <c r="H82" s="35"/>
     </row>
     <row r="83" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B83" s="75"/>
-      <c r="C83" s="51" t="s">
+      <c r="B83" s="71"/>
+      <c r="C83" s="37" t="s">
         <v>19</v>
       </c>
       <c r="D83" s="37">
@@ -3230,10 +3215,10 @@
       </c>
     </row>
     <row r="84" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H84" s="58"/>
+      <c r="H84" s="55"/>
     </row>
     <row r="85" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B85" s="76" t="s">
+      <c r="B85" s="72" t="s">
         <v>159</v>
       </c>
       <c r="C85" s="25" t="s">
@@ -3254,7 +3239,7 @@
       <c r="H85" s="40"/>
     </row>
     <row r="86" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B86" s="77"/>
+      <c r="B86" s="73"/>
       <c r="C86" s="15" t="s">
         <v>2</v>
       </c>
@@ -3275,7 +3260,7 @@
       </c>
     </row>
     <row r="87" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B87" s="77"/>
+      <c r="B87" s="73"/>
       <c r="C87" s="15" t="s">
         <v>9</v>
       </c>
@@ -3296,7 +3281,7 @@
       </c>
     </row>
     <row r="88" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B88" s="77"/>
+      <c r="B88" s="73"/>
       <c r="C88" s="15" t="s">
         <v>10</v>
       </c>
@@ -3309,7 +3294,7 @@
       <c r="H88" s="41"/>
     </row>
     <row r="89" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B89" s="77"/>
+      <c r="B89" s="73"/>
       <c r="C89" s="15" t="s">
         <v>11</v>
       </c>
@@ -3322,7 +3307,7 @@
       <c r="H89" s="28"/>
     </row>
     <row r="90" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B90" s="77"/>
+      <c r="B90" s="73"/>
       <c r="C90" s="15" t="s">
         <v>12</v>
       </c>
@@ -3335,7 +3320,7 @@
       <c r="H90" s="28"/>
     </row>
     <row r="91" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B91" s="77"/>
+      <c r="B91" s="73"/>
       <c r="C91" s="15" t="s">
         <v>13</v>
       </c>
@@ -3348,7 +3333,7 @@
       <c r="H91" s="28"/>
     </row>
     <row r="92" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B92" s="77"/>
+      <c r="B92" s="73"/>
       <c r="C92" s="15" t="s">
         <v>14</v>
       </c>
@@ -3361,7 +3346,7 @@
       <c r="H92" s="28"/>
     </row>
     <row r="93" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B93" s="77"/>
+      <c r="B93" s="73"/>
       <c r="C93" s="15" t="s">
         <v>15</v>
       </c>
@@ -3382,7 +3367,7 @@
       </c>
     </row>
     <row r="94" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B94" s="77"/>
+      <c r="B94" s="73"/>
       <c r="C94" s="15" t="s">
         <v>16</v>
       </c>
@@ -3395,7 +3380,7 @@
       <c r="H94" s="28"/>
     </row>
     <row r="95" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B95" s="77"/>
+      <c r="B95" s="73"/>
       <c r="C95" s="15" t="s">
         <v>18</v>
       </c>
@@ -3408,7 +3393,7 @@
       <c r="H95" s="28"/>
     </row>
     <row r="96" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="78"/>
+      <c r="B96" s="74"/>
       <c r="C96" s="29" t="s">
         <v>19</v>
       </c>
@@ -3430,17 +3415,17 @@
     </row>
     <row r="97" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F97" s="24"/>
-      <c r="H97" s="56"/>
+      <c r="H97" s="53"/>
     </row>
     <row r="98" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B98" s="73" t="s">
+      <c r="B98" s="69" t="s">
         <v>160</v>
       </c>
       <c r="C98" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D98" s="32" t="s">
-        <v>88</v>
+      <c r="D98" s="32">
+        <v>377</v>
       </c>
       <c r="E98" s="42" t="s">
         <v>84</v>
@@ -3448,18 +3433,18 @@
       <c r="F98" s="42" t="s">
         <v>146</v>
       </c>
-      <c r="G98" s="52" t="s">
+      <c r="G98" s="50" t="s">
         <v>291</v>
       </c>
       <c r="H98" s="43"/>
     </row>
     <row r="99" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B99" s="74"/>
+      <c r="B99" s="70"/>
       <c r="C99" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D99" s="18" t="s">
-        <v>88</v>
+      <c r="D99" s="18">
+        <v>377</v>
       </c>
       <c r="E99" s="19" t="s">
         <v>85</v>
@@ -3475,12 +3460,12 @@
       </c>
     </row>
     <row r="100" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B100" s="74"/>
+      <c r="B100" s="70"/>
       <c r="C100" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D100" s="18" t="s">
-        <v>88</v>
+      <c r="D100" s="18">
+        <v>378</v>
       </c>
       <c r="E100" s="19" t="s">
         <v>104</v>
@@ -3496,12 +3481,12 @@
       </c>
     </row>
     <row r="101" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B101" s="74"/>
+      <c r="B101" s="70"/>
       <c r="C101" s="18" t="s">
         <v>10</v>
       </c>
       <c r="D101" s="18" t="s">
-        <v>88</v>
+        <v>317</v>
       </c>
       <c r="E101" s="20" t="s">
         <v>308</v>
@@ -3517,7 +3502,7 @@
       </c>
     </row>
     <row r="102" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B102" s="74"/>
+      <c r="B102" s="70"/>
       <c r="C102" s="18" t="s">
         <v>11</v>
       </c>
@@ -3530,7 +3515,7 @@
       <c r="H102" s="36"/>
     </row>
     <row r="103" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B103" s="74"/>
+      <c r="B103" s="70"/>
       <c r="C103" s="18" t="s">
         <v>12</v>
       </c>
@@ -3543,7 +3528,7 @@
       <c r="H103" s="36"/>
     </row>
     <row r="104" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B104" s="74"/>
+      <c r="B104" s="70"/>
       <c r="C104" s="18" t="s">
         <v>13</v>
       </c>
@@ -3556,33 +3541,33 @@
       <c r="H104" s="36"/>
     </row>
     <row r="105" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B105" s="74"/>
+      <c r="B105" s="70"/>
       <c r="C105" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D105" s="18" t="s">
-        <v>88</v>
+      <c r="D105" s="18">
+        <v>393</v>
       </c>
       <c r="E105" s="20" t="s">
+        <v>311</v>
+      </c>
+      <c r="F105" s="20" t="s">
         <v>312</v>
-      </c>
-      <c r="F105" s="20" t="s">
-        <v>313</v>
       </c>
       <c r="G105" s="48" t="s">
         <v>244</v>
       </c>
       <c r="H105" s="36" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="106" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B106" s="74"/>
+      <c r="B106" s="70"/>
       <c r="C106" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D106" s="18" t="s">
-        <v>88</v>
+      <c r="D106" s="18">
+        <v>393</v>
       </c>
       <c r="E106" s="20" t="s">
         <v>105</v>
@@ -3598,28 +3583,28 @@
       </c>
     </row>
     <row r="107" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B107" s="74"/>
+      <c r="B107" s="70"/>
       <c r="C107" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D107" s="18" t="s">
-        <v>88</v>
+      <c r="D107" s="18">
+        <v>393</v>
       </c>
       <c r="E107" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="F107" s="20" t="s">
         <v>314</v>
-      </c>
-      <c r="F107" s="20" t="s">
-        <v>315</v>
       </c>
       <c r="G107" s="48" t="s">
         <v>246</v>
       </c>
       <c r="H107" s="36" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="108" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B108" s="74"/>
+      <c r="B108" s="70"/>
       <c r="C108" s="18" t="s">
         <v>18</v>
       </c>
@@ -3632,12 +3617,12 @@
       <c r="H108" s="36"/>
     </row>
     <row r="109" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B109" s="75"/>
+      <c r="B109" s="71"/>
       <c r="C109" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="D109" s="37" t="s">
-        <v>88</v>
+      <c r="D109" s="37">
+        <v>397</v>
       </c>
       <c r="E109" s="38" t="s">
         <v>256</v>
@@ -3692,35 +3677,35 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
     </row>
     <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="71"/>
-      <c r="D3" s="80" t="s">
+      <c r="C3" s="67"/>
+      <c r="D3" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="81"/>
-      <c r="F3" s="82"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="78"/>
     </row>
     <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="71"/>
-      <c r="D4" s="80" t="s">
+      <c r="C4" s="67"/>
+      <c r="D4" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="81"/>
-      <c r="F4" s="82"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="78"/>
     </row>
     <row r="5" spans="2:6" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>

</xml_diff>